<commit_message>
docs: add Wine UIs
</commit_message>
<xml_diff>
--- a/Settings/Install.xlsx
+++ b/Settings/Install.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markus/Projects/wiki/Settings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DEF0C7-71A9-E14E-9343-3136FA0FFD43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85506E8E-F558-4D49-92AE-F376D6FEAC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44800" yWindow="620" windowWidth="22400" windowHeight="27740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25600" yWindow="620" windowWidth="25600" windowHeight="31780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Windows" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="451">
   <si>
     <t>adblockpluschrome</t>
   </si>
@@ -1254,9 +1254,6 @@
     <t>https://heroicgameslauncher.com/downloads (Epic, GOG, Amazon)</t>
   </si>
   <si>
-    <t>Wine UI (Steam)</t>
-  </si>
-  <si>
     <t>https://www.golem.de/news/tools-fuer-das-game-porting-toolkit-windows-games-auf-dem-mac-spielen-2401-180913-3.html</t>
   </si>
   <si>
@@ -1446,10 +1443,22 @@
     <t>Meta Paket Tracker</t>
   </si>
   <si>
-    <t>Davinice Resolve</t>
-  </si>
-  <si>
     <t>Video Editor</t>
+  </si>
+  <si>
+    <t>Wine UI (Steam) - DEPRECATED</t>
+  </si>
+  <si>
+    <t>frankea/whisky/whisky</t>
+  </si>
+  <si>
+    <t>https://frankea.github.io/Whisky/</t>
+  </si>
+  <si>
+    <t>DaVinci Resolve</t>
+  </si>
+  <si>
+    <t>https://sikarugir.com/</t>
   </si>
 </sst>
 </file>
@@ -1978,10 +1987,10 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>429</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>69</v>
@@ -3205,7 +3214,7 @@
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
       <c r="H72" s="7" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
@@ -3335,7 +3344,7 @@
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="1"/>
       <c r="B80" s="13" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -4598,7 +4607,7 @@
         <v>297</v>
       </c>
       <c r="C33" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -4702,7 +4711,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F93F60-305A-704A-9194-4387AC0BEE7B}">
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
@@ -4724,7 +4733,7 @@
         <v>359</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -4810,7 +4819,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B8" t="s">
         <v>289</v>
@@ -4824,7 +4833,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B9" t="s">
         <v>289</v>
@@ -4849,7 +4858,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B11" t="s">
         <v>289</v>
@@ -4863,7 +4872,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B12" t="s">
         <v>297</v>
@@ -4872,7 +4881,7 @@
         <v>289</v>
       </c>
       <c r="D12" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -4886,7 +4895,7 @@
         <v>289</v>
       </c>
       <c r="D13" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -4944,12 +4953,12 @@
         <v>289</v>
       </c>
       <c r="D18" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B19" t="s">
         <v>297</v>
@@ -4958,12 +4967,12 @@
         <v>289</v>
       </c>
       <c r="D19" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B20" t="s">
         <v>289</v>
@@ -5030,16 +5039,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>397</v>
+      </c>
+      <c r="B25" t="s">
+        <v>289</v>
+      </c>
+      <c r="C25" t="s">
         <v>398</v>
       </c>
-      <c r="B25" t="s">
-        <v>289</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>399</v>
-      </c>
-      <c r="D25" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -5058,7 +5067,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B27" t="s">
         <v>289</v>
@@ -5109,7 +5118,7 @@
         <v>289</v>
       </c>
       <c r="D30" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -5142,18 +5151,18 @@
         <v>379</v>
       </c>
       <c r="B33" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="C33" t="s">
         <v>289</v>
       </c>
       <c r="D33" t="s">
-        <v>382</v>
+        <v>446</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>380</v>
+        <v>447</v>
       </c>
       <c r="B34" t="s">
         <v>289</v>
@@ -5162,37 +5171,34 @@
         <v>289</v>
       </c>
       <c r="D34" t="s">
-        <v>381</v>
+        <v>448</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>384</v>
-      </c>
-      <c r="B35" t="s">
-        <v>289</v>
-      </c>
       <c r="C35" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D35" t="s">
-        <v>386</v>
+        <v>450</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B36" t="s">
         <v>289</v>
       </c>
       <c r="C36" t="s">
         <v>289</v>
+      </c>
+      <c r="D36" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B37" t="s">
         <v>289</v>
@@ -5201,12 +5207,12 @@
         <v>297</v>
       </c>
       <c r="D37" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="B38" t="s">
         <v>289</v>
@@ -5217,21 +5223,21 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B39" t="s">
         <v>289</v>
       </c>
       <c r="C39" t="s">
-        <v>289</v>
-      </c>
-      <c r="E39" s="19" t="s">
-        <v>289</v>
+        <v>297</v>
+      </c>
+      <c r="D39" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="B40" t="s">
         <v>289</v>
@@ -5242,7 +5248,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B41" t="s">
         <v>289</v>
@@ -5250,49 +5256,52 @@
       <c r="C41" t="s">
         <v>289</v>
       </c>
-      <c r="D41" t="s">
-        <v>391</v>
+      <c r="E41" s="19" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>407</v>
+        <v>388</v>
       </c>
       <c r="B42" t="s">
         <v>289</v>
       </c>
       <c r="C42" t="s">
-        <v>297</v>
-      </c>
-      <c r="D42" t="s">
-        <v>441</v>
+        <v>289</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>408</v>
+        <v>389</v>
       </c>
       <c r="B43" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="C43" t="s">
         <v>289</v>
+      </c>
+      <c r="D43" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B44" t="s">
         <v>289</v>
       </c>
       <c r="C44" t="s">
-        <v>289</v>
+        <v>297</v>
+      </c>
+      <c r="D44" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="B45" t="s">
         <v>297</v>
@@ -5300,41 +5309,35 @@
       <c r="C45" t="s">
         <v>289</v>
       </c>
-      <c r="D45" t="s">
-        <v>413</v>
-      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B46" t="s">
         <v>289</v>
       </c>
       <c r="C46" t="s">
         <v>289</v>
-      </c>
-      <c r="D46" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="B47" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="C47" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D47" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>423</v>
+        <v>409</v>
       </c>
       <c r="B48" t="s">
         <v>289</v>
@@ -5343,26 +5346,26 @@
         <v>289</v>
       </c>
       <c r="D48" t="s">
-        <v>424</v>
+        <v>411</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="B49" t="s">
         <v>289</v>
       </c>
       <c r="C49" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="D49" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B50" t="s">
         <v>289</v>
@@ -5371,12 +5374,12 @@
         <v>289</v>
       </c>
       <c r="D50" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>431</v>
+        <v>424</v>
       </c>
       <c r="B51" t="s">
         <v>289</v>
@@ -5385,12 +5388,12 @@
         <v>289</v>
       </c>
       <c r="D51" t="s">
-        <v>432</v>
+        <v>425</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>433</v>
+        <v>426</v>
       </c>
       <c r="B52" t="s">
         <v>289</v>
@@ -5399,12 +5402,12 @@
         <v>289</v>
       </c>
       <c r="D52" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B53" t="s">
         <v>289</v>
@@ -5413,12 +5416,12 @@
         <v>289</v>
       </c>
       <c r="D53" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B54" t="s">
         <v>289</v>
@@ -5427,12 +5430,12 @@
         <v>289</v>
       </c>
       <c r="D54" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
       <c r="B55" t="s">
         <v>289</v>
@@ -5441,40 +5444,40 @@
         <v>289</v>
       </c>
       <c r="D55" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="B56" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="C56" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D56" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="B57" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="C57" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D57" t="s">
-        <v>445</v>
+        <v>438</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="B58" t="s">
         <v>297</v>
@@ -5483,20 +5486,48 @@
         <v>297</v>
       </c>
       <c r="D58" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="18"/>
+      <c r="A59" t="s">
+        <v>443</v>
+      </c>
+      <c r="B59" t="s">
+        <v>297</v>
+      </c>
+      <c r="C59" t="s">
+        <v>297</v>
+      </c>
+      <c r="D59" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="18" t="s">
-        <v>383</v>
+      <c r="A60" t="s">
+        <v>449</v>
+      </c>
+      <c r="B60" t="s">
+        <v>297</v>
+      </c>
+      <c r="C60" t="s">
+        <v>297</v>
+      </c>
+      <c r="D60" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="18"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="18" t="s">
+        <v>382</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A60" r:id="rId1" xr:uid="{65CB6B51-C990-C94E-8E20-9886EFDBDD52}"/>
+    <hyperlink ref="A62" r:id="rId1" xr:uid="{65CB6B51-C990-C94E-8E20-9886EFDBDD52}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -5519,10 +5550,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B2" t="s">
         <v>403</v>
-      </c>
-      <c r="B2" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -5532,12 +5563,12 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update Windows installed tools
</commit_message>
<xml_diff>
--- a/Settings/Install.xlsx
+++ b/Settings/Install.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markus/Projects/wiki/Settings/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\markus\projects\wiki\Settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24869C27-654C-3243-A2FB-8C2E15AB2500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B9A3EC-4D48-4A43-872D-1462CF10C177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="620" windowWidth="25600" windowHeight="31780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Windows" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="454">
   <si>
     <t>adblockpluschrome</t>
   </si>
@@ -654,9 +654,6 @@
     <t>Amazon.AWSCLI</t>
   </si>
   <si>
-    <t>dbeaver.dbeaver</t>
-  </si>
-  <si>
     <t>OliverBetz.ExifTool</t>
   </si>
   <si>
@@ -1462,6 +1459,15 @@
   </si>
   <si>
     <t>qrtool</t>
+  </si>
+  <si>
+    <t>dbeaver.dbeaver.community</t>
+  </si>
+  <si>
+    <t>In Logitech Options+ enthalten</t>
+  </si>
+  <si>
+    <t>Enthält LogiBolt</t>
   </si>
 </sst>
 </file>
@@ -1978,22 +1984,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H139"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="6.1640625" customWidth="1"/>
-    <col min="5" max="5" width="6.5" customWidth="1"/>
-    <col min="6" max="7" width="7.6640625" customWidth="1"/>
-    <col min="8" max="8" width="70.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="6.1796875" customWidth="1"/>
+    <col min="5" max="5" width="6.453125" customWidth="1"/>
+    <col min="6" max="7" width="7.6328125" customWidth="1"/>
+    <col min="8" max="8" width="70.6328125" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>428</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>429</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>69</v>
@@ -2014,7 +2020,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>57</v>
       </c>
@@ -2038,7 +2044,7 @@
       </c>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2054,7 +2060,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="13"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>58</v>
       </c>
@@ -2077,15 +2083,15 @@
         <v>54</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -2094,12 +2100,12 @@
       <c r="G5" s="3"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -2110,7 +2116,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>91</v>
       </c>
@@ -2124,7 +2130,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>92</v>
       </c>
@@ -2138,7 +2144,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>59</v>
       </c>
@@ -2158,7 +2164,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>98</v>
       </c>
@@ -2172,7 +2178,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
@@ -2184,7 +2190,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>112</v>
       </c>
@@ -2200,7 +2206,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>122</v>
       </c>
@@ -2214,7 +2220,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>123</v>
       </c>
@@ -2228,12 +2234,12 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -2241,10 +2247,10 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="11" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>136</v>
       </c>
@@ -2260,7 +2266,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>4</v>
       </c>
@@ -2272,12 +2278,12 @@
       <c r="G17" s="3"/>
       <c r="H17" s="7"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -2286,12 +2292,12 @@
       <c r="G18" s="3"/>
       <c r="H18" s="7"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>54</v>
@@ -2302,12 +2308,12 @@
       <c r="G19" s="3"/>
       <c r="H19" s="7"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>182</v>
+        <v>451</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>54</v>
@@ -2320,12 +2326,12 @@
       <c r="G20" s="3"/>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>54</v>
@@ -2336,12 +2342,12 @@
       <c r="G21" s="3"/>
       <c r="H21" s="7"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>171</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -2354,7 +2360,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>6</v>
       </c>
@@ -2370,7 +2376,7 @@
       <c r="G23" s="3"/>
       <c r="H23" s="7"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>7</v>
       </c>
@@ -2382,12 +2388,12 @@
       <c r="G24" s="3"/>
       <c r="H24" s="7"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>100</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>54</v>
@@ -2400,12 +2406,12 @@
       <c r="G25" s="3"/>
       <c r="H25" s="7"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>97</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>54</v>
@@ -2418,12 +2424,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>54</v>
@@ -2438,12 +2444,12 @@
       </c>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>54</v>
@@ -2457,15 +2463,15 @@
         <v>54</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
         <v>114</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>54</v>
@@ -2478,7 +2484,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>9</v>
       </c>
@@ -2498,12 +2504,12 @@
       <c r="G30" s="3"/>
       <c r="H30" s="7"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>54</v>
@@ -2520,12 +2526,12 @@
       <c r="G31" s="3"/>
       <c r="H31" s="7"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>54</v>
@@ -2540,12 +2546,12 @@
       </c>
       <c r="H32" s="7"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -2556,12 +2562,12 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>55</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>54</v>
@@ -2574,12 +2580,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>101</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -2590,12 +2596,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>54</v>
@@ -2608,12 +2614,12 @@
       <c r="G36" s="3"/>
       <c r="H36" s="7"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -2622,12 +2628,12 @@
       <c r="G37" s="3"/>
       <c r="H37" s="7"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>86</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>54</v>
@@ -2642,12 +2648,12 @@
         <v>130</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>54</v>
@@ -2664,12 +2670,12 @@
       <c r="G39" s="3"/>
       <c r="H39" s="7"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>54</v>
@@ -2682,7 +2688,7 @@
       <c r="G40" s="3"/>
       <c r="H40" s="7"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>14</v>
       </c>
@@ -2694,12 +2700,12 @@
       <c r="G41" s="3"/>
       <c r="H41" s="7"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -2710,7 +2716,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
         <v>83</v>
       </c>
@@ -2724,12 +2730,12 @@
         <v>84</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>54</v>
@@ -2740,12 +2746,12 @@
       <c r="G44" s="3"/>
       <c r="H44" s="7"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="12" t="s">
         <v>147</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -2760,12 +2766,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>54</v>
@@ -2782,12 +2788,12 @@
         <v>150</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>54</v>
@@ -2802,12 +2808,12 @@
       <c r="G47" s="3"/>
       <c r="H47" s="7"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
         <v>95</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>54</v>
@@ -2817,15 +2823,15 @@
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
       <c r="H48" s="11" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>54</v>
@@ -2838,12 +2844,12 @@
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -2854,7 +2860,7 @@
       <c r="G50" s="3"/>
       <c r="H50" s="7"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>18</v>
       </c>
@@ -2870,12 +2876,12 @@
       <c r="G51" s="3"/>
       <c r="H51" s="7"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>54</v>
@@ -2888,12 +2894,12 @@
       <c r="G52" s="3"/>
       <c r="H52" s="7"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -2902,12 +2908,12 @@
       <c r="G53" s="3"/>
       <c r="H53" s="7"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>54</v>
@@ -2924,12 +2930,12 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>54</v>
@@ -2944,12 +2950,12 @@
       </c>
       <c r="H55" s="7"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>160</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>54</v>
@@ -2966,7 +2972,7 @@
       </c>
       <c r="H56" s="7"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>21</v>
       </c>
@@ -2984,12 +2990,12 @@
       </c>
       <c r="H57" s="7"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>54</v>
@@ -3004,7 +3010,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="10" t="s">
         <v>22</v>
       </c>
@@ -3016,7 +3022,7 @@
       <c r="G59" s="3"/>
       <c r="H59" s="7"/>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>134</v>
       </c>
@@ -3030,12 +3036,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>120</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -3046,28 +3052,28 @@
         <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="1"/>
       <c r="B62" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D62" s="3"/>
-      <c r="E62" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E62" s="3"/>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
-      <c r="H62" s="7"/>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H62" s="7" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3" t="s">
@@ -3078,12 +3084,12 @@
       <c r="G63" s="3"/>
       <c r="H63" s="7"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B64" s="14" t="s">
         <v>228</v>
-      </c>
-      <c r="B64" s="14" t="s">
-        <v>229</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>54</v>
@@ -3094,9 +3100,11 @@
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
-      <c r="H64" s="7"/>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H64" s="7" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>23</v>
       </c>
@@ -3110,12 +3118,12 @@
       <c r="G65" s="3"/>
       <c r="H65" s="7"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
@@ -3126,12 +3134,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>139</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
@@ -3142,12 +3150,12 @@
         <v>141</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
@@ -3156,12 +3164,12 @@
       <c r="G68" s="3"/>
       <c r="H68" s="7"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
@@ -3170,12 +3178,12 @@
       <c r="G69" s="3"/>
       <c r="H69" s="7"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>54</v>
@@ -3188,12 +3196,12 @@
       <c r="G70" s="3"/>
       <c r="H70" s="7"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>106</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C71" s="3"/>
       <c r="D71" s="3"/>
@@ -3204,12 +3212,12 @@
       <c r="G71" s="3"/>
       <c r="H71" s="7"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C72" s="3"/>
       <c r="D72" s="3"/>
@@ -3217,15 +3225,15 @@
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
       <c r="H72" s="7" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C73" s="3"/>
       <c r="D73" s="3" t="s">
@@ -3238,12 +3246,12 @@
       </c>
       <c r="H73" s="7"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C74" s="3"/>
       <c r="D74" s="3"/>
@@ -3252,12 +3260,12 @@
       <c r="G74" s="3"/>
       <c r="H74" s="7"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="10" t="s">
         <v>176</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>54</v>
@@ -3268,12 +3276,12 @@
       <c r="G75" s="3"/>
       <c r="H75" s="7"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>54</v>
@@ -3286,12 +3294,12 @@
       <c r="G76" s="3"/>
       <c r="H76" s="7"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>54</v>
@@ -3302,22 +3310,16 @@
       <c r="G77" s="3"/>
       <c r="H77" s="7"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E78" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
       <c r="F78" s="3" t="s">
         <v>54</v>
       </c>
@@ -3326,12 +3328,12 @@
       </c>
       <c r="H78" s="7"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
@@ -3344,10 +3346,10 @@
         <v>151</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="1"/>
       <c r="B80" s="13" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
@@ -3358,12 +3360,12 @@
       <c r="G80" s="3"/>
       <c r="H80" s="7"/>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
@@ -3372,7 +3374,7 @@
       <c r="G81" s="3"/>
       <c r="H81" s="7"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>94</v>
       </c>
@@ -3386,12 +3388,12 @@
       <c r="G82" s="3"/>
       <c r="H82" s="7"/>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
@@ -3400,12 +3402,12 @@
       <c r="G83" s="3"/>
       <c r="H83" s="7"/>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
@@ -3414,28 +3416,26 @@
       <c r="G84" s="3"/>
       <c r="H84" s="7"/>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
-      <c r="E85" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E85" s="3"/>
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
       <c r="H85" s="7"/>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
@@ -3444,12 +3444,12 @@
       <c r="G86" s="3"/>
       <c r="H86" s="7"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>177</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>54</v>
@@ -3462,12 +3462,12 @@
       <c r="G87" s="3"/>
       <c r="H87" s="7"/>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>54</v>
@@ -3484,12 +3484,12 @@
       </c>
       <c r="H88" s="7"/>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>54</v>
@@ -3502,12 +3502,12 @@
       <c r="G89" s="3"/>
       <c r="H89" s="7"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>54</v>
@@ -3520,12 +3520,12 @@
       <c r="G90" s="3"/>
       <c r="H90" s="7"/>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
@@ -3534,12 +3534,12 @@
       <c r="G91" s="3"/>
       <c r="H91" s="7"/>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>54</v>
@@ -3550,12 +3550,12 @@
       <c r="G92" s="3"/>
       <c r="H92" s="7"/>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="10" t="s">
         <v>116</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>54</v>
@@ -3568,12 +3568,12 @@
         <v>117</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>54</v>
@@ -3586,12 +3586,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
@@ -3602,12 +3602,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>161</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>54</v>
@@ -3620,12 +3620,12 @@
         <v>162</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
@@ -3634,7 +3634,7 @@
       <c r="G97" s="3"/>
       <c r="H97" s="7"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>81</v>
       </c>
@@ -3646,12 +3646,12 @@
       <c r="G98" s="3"/>
       <c r="H98" s="7"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B99" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
@@ -3662,12 +3662,12 @@
       <c r="G99" s="3"/>
       <c r="H99" s="7"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
@@ -3676,12 +3676,12 @@
       <c r="G100" s="3"/>
       <c r="H100" s="7"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B101" s="13" t="s">
         <v>285</v>
-      </c>
-      <c r="B101" s="13" t="s">
-        <v>286</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>54</v>
@@ -3692,12 +3692,12 @@
       <c r="G101" s="3"/>
       <c r="H101" s="7"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="10" t="s">
         <v>118</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>54</v>
@@ -3710,12 +3710,12 @@
         <v>119</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>54</v>
@@ -3728,12 +3728,12 @@
       <c r="G103" s="3"/>
       <c r="H103" s="7"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
@@ -3742,12 +3742,12 @@
       <c r="G104" s="3"/>
       <c r="H104" s="7"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C105" s="3"/>
       <c r="D105" s="3"/>
@@ -3758,12 +3758,12 @@
         <v>154</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B106" s="13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>54</v>
@@ -3776,12 +3776,12 @@
       <c r="G106" s="3"/>
       <c r="H106" s="7"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B107" s="13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>54</v>
@@ -3794,68 +3794,62 @@
       <c r="G107" s="3"/>
       <c r="H107" s="7"/>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>169</v>
       </c>
       <c r="B108" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
-      <c r="E108" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E108" s="3"/>
       <c r="F108" s="3"/>
       <c r="G108" s="3"/>
       <c r="H108" s="7" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>170</v>
       </c>
       <c r="B109" s="13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
-      <c r="E109" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E109" s="3"/>
       <c r="F109" s="3"/>
       <c r="G109" s="3"/>
       <c r="H109" s="7" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>165</v>
       </c>
       <c r="B110" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D110" s="3"/>
-      <c r="E110" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E110" s="3"/>
       <c r="F110" s="3"/>
       <c r="G110" s="3"/>
       <c r="H110" s="7" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B111" s="13" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
@@ -3866,12 +3860,12 @@
       <c r="G111" s="3"/>
       <c r="H111" s="7"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B112" s="13" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
@@ -3880,7 +3874,7 @@
       <c r="G112" s="3"/>
       <c r="H112" s="7"/>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>67</v>
       </c>
@@ -3894,12 +3888,12 @@
         <v>175</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B114" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>54</v>
@@ -3907,21 +3901,19 @@
       <c r="D114" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E114" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="E114" s="3"/>
       <c r="F114" s="3"/>
       <c r="G114" s="3"/>
       <c r="H114" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="10" t="s">
         <v>87</v>
       </c>
       <c r="B115" s="13" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>54</v>
@@ -3934,7 +3926,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>42</v>
       </c>
@@ -3950,12 +3942,12 @@
       <c r="G116" s="3"/>
       <c r="H116" s="7"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B117" s="13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>54</v>
@@ -3968,12 +3960,12 @@
       <c r="G117" s="3"/>
       <c r="H117" s="7"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B118" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
@@ -3982,12 +3974,12 @@
       <c r="G118" s="3"/>
       <c r="H118" s="7"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B119" s="13" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
@@ -3996,12 +3988,12 @@
       <c r="G119" s="3"/>
       <c r="H119" s="7"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B120" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>54</v>
@@ -4018,12 +4010,12 @@
       </c>
       <c r="H120" s="7"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B121" s="13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>54</v>
@@ -4034,12 +4026,12 @@
       <c r="G121" s="3"/>
       <c r="H121" s="7"/>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B122" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>54</v>
@@ -4054,12 +4046,12 @@
       <c r="G122" s="3"/>
       <c r="H122" s="7"/>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B123" s="13" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
@@ -4068,7 +4060,7 @@
       <c r="G123" s="3"/>
       <c r="H123" s="7"/>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>163</v>
       </c>
@@ -4084,7 +4076,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>72</v>
       </c>
@@ -4102,12 +4094,12 @@
         <v>152</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B126" s="13" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>54</v>
@@ -4126,12 +4118,12 @@
         <v>145</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B127" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>54</v>
@@ -4146,12 +4138,12 @@
       <c r="G127" s="3"/>
       <c r="H127" s="7"/>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B128" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>54</v>
@@ -4164,12 +4156,12 @@
       <c r="G128" s="3"/>
       <c r="H128" s="7"/>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>110</v>
       </c>
       <c r="B129" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
@@ -4178,7 +4170,7 @@
       <c r="G129" s="3"/>
       <c r="H129" s="7"/>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="8" t="s">
         <v>125</v>
       </c>
@@ -4190,7 +4182,7 @@
       <c r="G130" s="3"/>
       <c r="H130" s="7"/>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" s="9" t="s">
         <v>126</v>
       </c>
@@ -4202,12 +4194,12 @@
       <c r="G131" s="3"/>
       <c r="H131" s="7"/>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B132" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
@@ -4218,7 +4210,7 @@
       <c r="G132" s="3"/>
       <c r="H132" s="7"/>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>52</v>
       </c>
@@ -4234,12 +4226,12 @@
       <c r="G133" s="3"/>
       <c r="H133" s="7"/>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="10" t="s">
         <v>53</v>
       </c>
       <c r="B134" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>54</v>
@@ -4252,12 +4244,12 @@
       <c r="G134" s="3"/>
       <c r="H134" s="7"/>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B135" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C135" s="3" t="s">
         <v>54</v>
@@ -4272,17 +4264,17 @@
       </c>
       <c r="H135" s="7"/>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="10" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="8" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="9" t="s">
         <v>127</v>
       </c>
@@ -4302,409 +4294,409 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="51" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>290</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="C1" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>292</v>
       </c>
-      <c r="D1" s="15" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>294</v>
       </c>
-      <c r="B2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>288</v>
+      </c>
+      <c r="C3" t="s">
+        <v>373</v>
+      </c>
+      <c r="D3" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>295</v>
       </c>
-      <c r="B3" t="s">
-        <v>289</v>
-      </c>
-      <c r="C3" t="s">
-        <v>374</v>
-      </c>
-      <c r="D3" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>296</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>297</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>299</v>
       </c>
-      <c r="B5" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C6" t="s">
         <v>300</v>
       </c>
-      <c r="B6" t="s">
-        <v>297</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>301</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>303</v>
       </c>
-      <c r="B7" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>304</v>
       </c>
-      <c r="B8" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>305</v>
       </c>
-      <c r="B9" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>306</v>
       </c>
-      <c r="B10" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>307</v>
       </c>
-      <c r="B11" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>308</v>
       </c>
-      <c r="B12" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>309</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>311</v>
       </c>
-      <c r="B14" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>312</v>
       </c>
-      <c r="B15" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>313</v>
       </c>
-      <c r="B16" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>314</v>
       </c>
-      <c r="B17" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>315</v>
       </c>
-      <c r="B18" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
         <v>316</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
+        <v>288</v>
+      </c>
+      <c r="D20" t="s">
         <v>318</v>
       </c>
-      <c r="B20" t="s">
-        <v>289</v>
-      </c>
-      <c r="D20" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>320</v>
       </c>
-      <c r="B21" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>321</v>
       </c>
-      <c r="B22" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>322</v>
       </c>
-      <c r="B23" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>323</v>
       </c>
-      <c r="B24" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>324</v>
       </c>
-      <c r="B25" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="B26" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>325</v>
       </c>
-      <c r="B26" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="B27" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="C27" t="s">
         <v>326</v>
       </c>
-      <c r="B27" s="16" t="s">
-        <v>297</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>327</v>
       </c>
-      <c r="D27" t="s">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>329</v>
       </c>
-      <c r="B28" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
+        <v>296</v>
+      </c>
+      <c r="C29" t="s">
         <v>330</v>
       </c>
-      <c r="B29" t="s">
-        <v>297</v>
-      </c>
-      <c r="C29" t="s">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="B30" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>332</v>
       </c>
-      <c r="B30" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>333</v>
       </c>
-      <c r="B31" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
+        <v>296</v>
+      </c>
+      <c r="C32" t="s">
         <v>334</v>
       </c>
-      <c r="B32" t="s">
-        <v>297</v>
-      </c>
-      <c r="C32" t="s">
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
+        <v>296</v>
+      </c>
+      <c r="C33" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>336</v>
       </c>
-      <c r="B33" t="s">
-        <v>297</v>
-      </c>
-      <c r="C33" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
+        <v>296</v>
+      </c>
+      <c r="C34" t="s">
         <v>337</v>
       </c>
-      <c r="B34" t="s">
-        <v>297</v>
-      </c>
-      <c r="C34" t="s">
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
+        <v>296</v>
+      </c>
+      <c r="C35" t="s">
         <v>339</v>
       </c>
-      <c r="B35" t="s">
-        <v>297</v>
-      </c>
-      <c r="C35" t="s">
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>341</v>
       </c>
-      <c r="B36" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>342</v>
       </c>
-      <c r="B37" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>343</v>
       </c>
-      <c r="B38" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>344</v>
       </c>
-      <c r="B39" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="B40" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>345</v>
       </c>
-      <c r="B40" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="B41" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>346</v>
       </c>
-      <c r="B41" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="B42" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>347</v>
       </c>
-      <c r="B42" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="B43" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>348</v>
       </c>
-      <c r="B43" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>349</v>
-      </c>
       <c r="B44" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -4715,828 +4707,828 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F93F60-305A-704A-9194-4387AC0BEE7B}">
   <dimension ref="A1:E63"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="66.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>357</v>
       </c>
-      <c r="B1" s="17" t="s">
-        <v>373</v>
-      </c>
-      <c r="C1" s="17" t="s">
+      <c r="D1" s="17" t="s">
         <v>358</v>
       </c>
-      <c r="D1" s="17" t="s">
-        <v>359</v>
-      </c>
       <c r="E1" s="17" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C2" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E3" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B4" t="s">
+        <v>288</v>
+      </c>
+      <c r="C4" t="s">
+        <v>296</v>
+      </c>
+      <c r="D4" t="s">
         <v>350</v>
       </c>
-      <c r="B4" t="s">
-        <v>289</v>
-      </c>
-      <c r="C4" t="s">
-        <v>297</v>
-      </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>288</v>
+      </c>
+      <c r="C5" t="s">
+        <v>288</v>
+      </c>
+      <c r="D5" t="s">
         <v>352</v>
       </c>
-      <c r="B5" t="s">
-        <v>289</v>
-      </c>
-      <c r="C5" t="s">
-        <v>289</v>
-      </c>
-      <c r="D5" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E6" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D7" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>390</v>
+      </c>
+      <c r="B8" t="s">
+        <v>288</v>
+      </c>
+      <c r="C8" t="s">
+        <v>288</v>
+      </c>
+      <c r="D8" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>391</v>
       </c>
-      <c r="B8" t="s">
-        <v>289</v>
-      </c>
-      <c r="C8" t="s">
-        <v>289</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="B9" t="s">
+        <v>288</v>
+      </c>
+      <c r="C9" t="s">
+        <v>288</v>
+      </c>
+      <c r="E9" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B10" t="s">
+        <v>288</v>
+      </c>
+      <c r="C10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>392</v>
       </c>
-      <c r="B9" t="s">
-        <v>289</v>
-      </c>
-      <c r="C9" t="s">
-        <v>289</v>
-      </c>
-      <c r="E9" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>356</v>
-      </c>
-      <c r="B10" t="s">
-        <v>289</v>
-      </c>
-      <c r="C10" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>393</v>
-      </c>
       <c r="B11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E11" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>417</v>
+      </c>
+      <c r="B12" t="s">
+        <v>296</v>
+      </c>
+      <c r="C12" t="s">
+        <v>288</v>
+      </c>
+      <c r="D12" t="s">
         <v>418</v>
       </c>
-      <c r="B12" t="s">
-        <v>297</v>
-      </c>
-      <c r="C12" t="s">
-        <v>289</v>
-      </c>
-      <c r="D12" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D13" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C14" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C15" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C16" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C17" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>360</v>
+      </c>
+      <c r="B18" t="s">
+        <v>288</v>
+      </c>
+      <c r="C18" t="s">
+        <v>288</v>
+      </c>
+      <c r="D18" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>395</v>
+      </c>
+      <c r="B19" t="s">
+        <v>296</v>
+      </c>
+      <c r="C19" t="s">
+        <v>288</v>
+      </c>
+      <c r="D19" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>394</v>
+      </c>
+      <c r="B20" t="s">
+        <v>288</v>
+      </c>
+      <c r="C20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>347</v>
+      </c>
+      <c r="B21" t="s">
+        <v>288</v>
+      </c>
+      <c r="C21" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>361</v>
       </c>
-      <c r="B18" t="s">
-        <v>289</v>
-      </c>
-      <c r="C18" t="s">
-        <v>289</v>
-      </c>
-      <c r="D18" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B22" t="s">
+        <v>288</v>
+      </c>
+      <c r="C22" t="s">
+        <v>296</v>
+      </c>
+      <c r="E22" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>362</v>
+      </c>
+      <c r="B23" t="s">
+        <v>288</v>
+      </c>
+      <c r="C23" t="s">
+        <v>296</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>364</v>
+      </c>
+      <c r="B24" t="s">
+        <v>288</v>
+      </c>
+      <c r="C24" t="s">
+        <v>296</v>
+      </c>
+      <c r="D24" t="s">
+        <v>363</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>396</v>
       </c>
-      <c r="B19" t="s">
-        <v>297</v>
-      </c>
-      <c r="C19" t="s">
-        <v>289</v>
-      </c>
-      <c r="D19" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>395</v>
-      </c>
-      <c r="B20" t="s">
-        <v>289</v>
-      </c>
-      <c r="C20" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>348</v>
-      </c>
-      <c r="B21" t="s">
-        <v>289</v>
-      </c>
-      <c r="C21" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>362</v>
-      </c>
-      <c r="B22" t="s">
-        <v>289</v>
-      </c>
-      <c r="C22" t="s">
-        <v>297</v>
-      </c>
-      <c r="E22" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>363</v>
-      </c>
-      <c r="B23" t="s">
-        <v>289</v>
-      </c>
-      <c r="C23" t="s">
-        <v>297</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="B25" t="s">
+        <v>288</v>
+      </c>
+      <c r="C25" t="s">
+        <v>397</v>
+      </c>
+      <c r="D25" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>365</v>
       </c>
-      <c r="B24" t="s">
-        <v>289</v>
-      </c>
-      <c r="C24" t="s">
-        <v>297</v>
-      </c>
-      <c r="D24" t="s">
-        <v>364</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>397</v>
-      </c>
-      <c r="B25" t="s">
-        <v>289</v>
-      </c>
-      <c r="C25" t="s">
-        <v>398</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="B26" t="s">
+        <v>288</v>
+      </c>
+      <c r="C26" t="s">
+        <v>288</v>
+      </c>
+      <c r="D26" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>366</v>
-      </c>
-      <c r="B26" t="s">
-        <v>289</v>
-      </c>
-      <c r="C26" t="s">
-        <v>289</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="B27" t="s">
+        <v>288</v>
+      </c>
+      <c r="C27" t="s">
+        <v>288</v>
+      </c>
+      <c r="D27" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>400</v>
-      </c>
-      <c r="B27" t="s">
-        <v>289</v>
-      </c>
-      <c r="C27" t="s">
-        <v>289</v>
-      </c>
-      <c r="D27" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="B28" t="s">
+        <v>288</v>
+      </c>
+      <c r="C28" t="s">
+        <v>296</v>
+      </c>
+      <c r="D28" t="s">
         <v>369</v>
       </c>
-      <c r="B28" t="s">
-        <v>289</v>
-      </c>
-      <c r="C28" t="s">
-        <v>297</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="E28" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>370</v>
       </c>
-      <c r="E28" s="19" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="B29" t="s">
+        <v>288</v>
+      </c>
+      <c r="C29" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>371</v>
       </c>
-      <c r="B29" t="s">
-        <v>289</v>
-      </c>
-      <c r="C29" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>372</v>
-      </c>
       <c r="B30" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C30" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D30" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C31" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>375</v>
+      </c>
+      <c r="B32" t="s">
+        <v>288</v>
+      </c>
+      <c r="C32" t="s">
+        <v>288</v>
+      </c>
+      <c r="D32" t="s">
         <v>376</v>
       </c>
-      <c r="B32" t="s">
-        <v>289</v>
-      </c>
-      <c r="C32" t="s">
-        <v>289</v>
-      </c>
-      <c r="D32" t="s">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>378</v>
+      </c>
+      <c r="B33" t="s">
+        <v>296</v>
+      </c>
+      <c r="C33" t="s">
+        <v>288</v>
+      </c>
+      <c r="D33" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>446</v>
+      </c>
+      <c r="B34" t="s">
+        <v>288</v>
+      </c>
+      <c r="C34" t="s">
+        <v>288</v>
+      </c>
+      <c r="D34" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C35" t="s">
+        <v>288</v>
+      </c>
+      <c r="D35" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>379</v>
+      </c>
+      <c r="B36" t="s">
+        <v>288</v>
+      </c>
+      <c r="C36" t="s">
+        <v>288</v>
+      </c>
+      <c r="D36" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>382</v>
+      </c>
+      <c r="B37" t="s">
+        <v>288</v>
+      </c>
+      <c r="C37" t="s">
+        <v>296</v>
+      </c>
+      <c r="D37" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>379</v>
-      </c>
-      <c r="B33" t="s">
-        <v>297</v>
-      </c>
-      <c r="C33" t="s">
-        <v>289</v>
-      </c>
-      <c r="D33" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>447</v>
-      </c>
-      <c r="B34" t="s">
-        <v>289</v>
-      </c>
-      <c r="C34" t="s">
-        <v>289</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="B38" t="s">
+        <v>288</v>
+      </c>
+      <c r="C38" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>383</v>
+      </c>
+      <c r="B39" t="s">
+        <v>288</v>
+      </c>
+      <c r="C39" t="s">
+        <v>296</v>
+      </c>
+      <c r="D39" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>385</v>
+      </c>
+      <c r="B40" t="s">
+        <v>288</v>
+      </c>
+      <c r="C40" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>386</v>
+      </c>
+      <c r="B41" t="s">
+        <v>288</v>
+      </c>
+      <c r="C41" t="s">
+        <v>288</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>387</v>
+      </c>
+      <c r="B42" t="s">
+        <v>288</v>
+      </c>
+      <c r="C42" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>388</v>
+      </c>
+      <c r="B43" t="s">
+        <v>288</v>
+      </c>
+      <c r="C43" t="s">
+        <v>288</v>
+      </c>
+      <c r="D43" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>405</v>
+      </c>
+      <c r="B44" t="s">
+        <v>288</v>
+      </c>
+      <c r="C44" t="s">
+        <v>296</v>
+      </c>
+      <c r="D44" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>406</v>
+      </c>
+      <c r="B45" t="s">
+        <v>296</v>
+      </c>
+      <c r="C45" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>407</v>
+      </c>
+      <c r="B46" t="s">
+        <v>288</v>
+      </c>
+      <c r="C46" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>409</v>
+      </c>
+      <c r="B47" t="s">
+        <v>296</v>
+      </c>
+      <c r="C47" t="s">
+        <v>288</v>
+      </c>
+      <c r="D47" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>408</v>
+      </c>
+      <c r="B48" t="s">
+        <v>288</v>
+      </c>
+      <c r="C48" t="s">
+        <v>288</v>
+      </c>
+      <c r="D48" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>413</v>
+      </c>
+      <c r="B49" t="s">
+        <v>288</v>
+      </c>
+      <c r="C49" t="s">
+        <v>296</v>
+      </c>
+      <c r="D49" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>421</v>
+      </c>
+      <c r="B50" t="s">
+        <v>288</v>
+      </c>
+      <c r="C50" t="s">
+        <v>288</v>
+      </c>
+      <c r="D50" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>423</v>
+      </c>
+      <c r="B51" t="s">
+        <v>288</v>
+      </c>
+      <c r="C51" t="s">
+        <v>288</v>
+      </c>
+      <c r="D51" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>425</v>
+      </c>
+      <c r="B52" t="s">
+        <v>288</v>
+      </c>
+      <c r="C52" t="s">
+        <v>288</v>
+      </c>
+      <c r="D52" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>429</v>
+      </c>
+      <c r="B53" t="s">
+        <v>288</v>
+      </c>
+      <c r="C53" t="s">
+        <v>288</v>
+      </c>
+      <c r="D53" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>431</v>
+      </c>
+      <c r="B54" t="s">
+        <v>288</v>
+      </c>
+      <c r="C54" t="s">
+        <v>288</v>
+      </c>
+      <c r="D54" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>433</v>
+      </c>
+      <c r="B55" t="s">
+        <v>288</v>
+      </c>
+      <c r="C55" t="s">
+        <v>288</v>
+      </c>
+      <c r="D55" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>435</v>
+      </c>
+      <c r="B56" t="s">
+        <v>288</v>
+      </c>
+      <c r="C56" t="s">
+        <v>288</v>
+      </c>
+      <c r="D56" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>438</v>
+      </c>
+      <c r="B57" t="s">
+        <v>288</v>
+      </c>
+      <c r="C57" t="s">
+        <v>288</v>
+      </c>
+      <c r="D57" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>440</v>
+      </c>
+      <c r="B58" t="s">
+        <v>296</v>
+      </c>
+      <c r="C58" t="s">
+        <v>296</v>
+      </c>
+      <c r="D58" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>442</v>
+      </c>
+      <c r="B59" t="s">
+        <v>296</v>
+      </c>
+      <c r="C59" t="s">
+        <v>296</v>
+      </c>
+      <c r="D59" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>448</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
-        <v>289</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="B60" t="s">
+        <v>296</v>
+      </c>
+      <c r="C60" t="s">
+        <v>296</v>
+      </c>
+      <c r="D60" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>380</v>
-      </c>
-      <c r="B36" t="s">
-        <v>289</v>
-      </c>
-      <c r="C36" t="s">
-        <v>289</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="B61" t="s">
+        <v>288</v>
+      </c>
+      <c r="C61" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="18"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="18" t="s">
         <v>381</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>383</v>
-      </c>
-      <c r="B37" t="s">
-        <v>289</v>
-      </c>
-      <c r="C37" t="s">
-        <v>297</v>
-      </c>
-      <c r="D37" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>378</v>
-      </c>
-      <c r="B38" t="s">
-        <v>289</v>
-      </c>
-      <c r="C38" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>384</v>
-      </c>
-      <c r="B39" t="s">
-        <v>289</v>
-      </c>
-      <c r="C39" t="s">
-        <v>297</v>
-      </c>
-      <c r="D39" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>386</v>
-      </c>
-      <c r="B40" t="s">
-        <v>289</v>
-      </c>
-      <c r="C40" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>387</v>
-      </c>
-      <c r="B41" t="s">
-        <v>289</v>
-      </c>
-      <c r="C41" t="s">
-        <v>289</v>
-      </c>
-      <c r="E41" s="19" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>388</v>
-      </c>
-      <c r="B42" t="s">
-        <v>289</v>
-      </c>
-      <c r="C42" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>389</v>
-      </c>
-      <c r="B43" t="s">
-        <v>289</v>
-      </c>
-      <c r="C43" t="s">
-        <v>289</v>
-      </c>
-      <c r="D43" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>406</v>
-      </c>
-      <c r="B44" t="s">
-        <v>289</v>
-      </c>
-      <c r="C44" t="s">
-        <v>297</v>
-      </c>
-      <c r="D44" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>407</v>
-      </c>
-      <c r="B45" t="s">
-        <v>297</v>
-      </c>
-      <c r="C45" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>408</v>
-      </c>
-      <c r="B46" t="s">
-        <v>289</v>
-      </c>
-      <c r="C46" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>410</v>
-      </c>
-      <c r="B47" t="s">
-        <v>297</v>
-      </c>
-      <c r="C47" t="s">
-        <v>289</v>
-      </c>
-      <c r="D47" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>409</v>
-      </c>
-      <c r="B48" t="s">
-        <v>289</v>
-      </c>
-      <c r="C48" t="s">
-        <v>289</v>
-      </c>
-      <c r="D48" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>414</v>
-      </c>
-      <c r="B49" t="s">
-        <v>289</v>
-      </c>
-      <c r="C49" t="s">
-        <v>297</v>
-      </c>
-      <c r="D49" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>422</v>
-      </c>
-      <c r="B50" t="s">
-        <v>289</v>
-      </c>
-      <c r="C50" t="s">
-        <v>289</v>
-      </c>
-      <c r="D50" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>424</v>
-      </c>
-      <c r="B51" t="s">
-        <v>289</v>
-      </c>
-      <c r="C51" t="s">
-        <v>289</v>
-      </c>
-      <c r="D51" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>426</v>
-      </c>
-      <c r="B52" t="s">
-        <v>289</v>
-      </c>
-      <c r="C52" t="s">
-        <v>289</v>
-      </c>
-      <c r="D52" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>430</v>
-      </c>
-      <c r="B53" t="s">
-        <v>289</v>
-      </c>
-      <c r="C53" t="s">
-        <v>289</v>
-      </c>
-      <c r="D53" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>432</v>
-      </c>
-      <c r="B54" t="s">
-        <v>289</v>
-      </c>
-      <c r="C54" t="s">
-        <v>289</v>
-      </c>
-      <c r="D54" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>434</v>
-      </c>
-      <c r="B55" t="s">
-        <v>289</v>
-      </c>
-      <c r="C55" t="s">
-        <v>289</v>
-      </c>
-      <c r="D55" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>436</v>
-      </c>
-      <c r="B56" t="s">
-        <v>289</v>
-      </c>
-      <c r="C56" t="s">
-        <v>289</v>
-      </c>
-      <c r="D56" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>439</v>
-      </c>
-      <c r="B57" t="s">
-        <v>289</v>
-      </c>
-      <c r="C57" t="s">
-        <v>289</v>
-      </c>
-      <c r="D57" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>441</v>
-      </c>
-      <c r="B58" t="s">
-        <v>297</v>
-      </c>
-      <c r="C58" t="s">
-        <v>297</v>
-      </c>
-      <c r="D58" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>443</v>
-      </c>
-      <c r="B59" t="s">
-        <v>297</v>
-      </c>
-      <c r="C59" t="s">
-        <v>297</v>
-      </c>
-      <c r="D59" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>449</v>
-      </c>
-      <c r="B60" t="s">
-        <v>297</v>
-      </c>
-      <c r="C60" t="s">
-        <v>297</v>
-      </c>
-      <c r="D60" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>451</v>
-      </c>
-      <c r="B61" t="s">
-        <v>289</v>
-      </c>
-      <c r="C61" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="18"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="18" t="s">
-        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -5551,38 +5543,38 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065AFD5E-E7C4-4344-BCB5-48CFA86F7E2C}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="63" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B2" t="s">
         <v>402</v>
       </c>
-      <c r="B2" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>